<commit_message>
Update testdata JSONs and Ingestion.xlsx from latest test run
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ingestion.xlsx
+++ b/Ingestion.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>BU</t>
   </si>
@@ -63,7 +63,7 @@
     <t>MHCA Approval_ARB</t>
   </si>
   <si>
-    <t>UNV3</t>
+    <t>CA</t>
   </si>
   <si>
     <t>ALL</t>
@@ -79,9 +79,6 @@
   </si>
   <si>
     <t>MAPD Multiple Claim ACK LTR</t>
-  </si>
-  <si>
-    <t>CA</t>
   </si>
   <si>
     <t>MAPD Multiple Claim ACK LTR.docx</t>
@@ -503,7 +500,7 @@
         <v>20</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>16</v>
@@ -512,7 +509,7 @@
         <v>17</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">

</xml_diff>